<commit_message>
docs: marcar CP-001, CP-002, CP-007 y CP-008 como Pasa
</commit_message>
<xml_diff>
--- a/docs/Plantilla_Casos_de_Prueba_S7.xlsx
+++ b/docs/Plantilla_Casos_de_Prueba_S7.xlsx
@@ -672,7 +672,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pasa</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pasa</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pasa</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pasa</t>
         </is>
       </c>
     </row>

</xml_diff>